<commit_message>
up to runo 20 part 1
</commit_message>
<xml_diff>
--- a/sources/translations_eng/translations.xlsx
+++ b/sources/translations_eng/translations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\karol\Desktop\new_github\claudevala\sources\translations_eng\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00612A4B-CC1C-435C-8FDA-A203306B8551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94901640-B4BC-498A-ABB0-AE4D0283BD97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3557FE8A-D42F-43F9-98C8-912E5CD1CDE3}"/>
   </bookViews>
@@ -337,22 +337,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -681,39 +676,37 @@
     <col min="5" max="16384" width="14.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:4" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:4" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="6">
         <v>1846</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="4" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-    </row>
+    <row r="3" spans="1:4" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="2">
@@ -727,7 +720,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2">
@@ -741,7 +734,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -755,7 +748,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -769,7 +762,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -783,7 +776,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" t="s">
         <v>0</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -797,7 +790,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -811,7 +804,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="A11" t="s">
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
@@ -825,7 +818,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" t="s">
         <v>0</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -839,7 +832,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
         <v>0</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -853,7 +846,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="2">
@@ -867,7 +860,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="A15" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="2">
@@ -881,7 +874,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="A16" t="s">
         <v>0</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -895,7 +888,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="A17" t="s">
         <v>0</v>
       </c>
       <c r="B17" s="2">
@@ -909,7 +902,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A18" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="2">

</xml_diff>